<commit_message>
VWAP mensuel mis à jour
</commit_message>
<xml_diff>
--- a/Nexans_VWAP.xlsx
+++ b/Nexans_VWAP.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="2026-06" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="VWAP_Mensuel" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2026-05" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,8 +19,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -50,9 +51,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -132,6 +134,23 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_202606" displayName="Table_202606" ref="A1:H23" headerRowCount="1">
   <autoFilter ref="A1:H23"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Date"/>
+    <tableColumn id="2" name="Adj Close"/>
+    <tableColumn id="3" name="Close"/>
+    <tableColumn id="4" name="High"/>
+    <tableColumn id="5" name="Low"/>
+    <tableColumn id="6" name="Open"/>
+    <tableColumn id="7" name="Volume"/>
+    <tableColumn id="8" name="VWAP"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_202605" displayName="Table_202605" ref="A1:H21" headerRowCount="1">
+  <autoFilter ref="A1:H21"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="Adj Close"/>
@@ -481,7 +500,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="B2" t="n">
@@ -507,7 +526,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>46175</v>
       </c>
       <c r="B3" t="n">
@@ -533,7 +552,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="B4" t="n">
@@ -559,7 +578,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>46177</v>
       </c>
       <c r="B5" t="n">
@@ -585,7 +604,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>46178</v>
       </c>
       <c r="B6" t="n">
@@ -611,7 +630,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>46181</v>
       </c>
       <c r="B7" t="n">
@@ -637,7 +656,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="B8" t="n">
@@ -663,7 +682,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="B9" t="n">
@@ -689,7 +708,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>46184</v>
       </c>
       <c r="B10" t="n">
@@ -715,7 +734,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="B11" t="n">
@@ -741,7 +760,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="B12" t="n">
@@ -767,7 +786,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>46189</v>
       </c>
       <c r="B13" t="n">
@@ -793,7 +812,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>46190</v>
       </c>
       <c r="B14" t="n">
@@ -819,7 +838,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="B15" t="n">
@@ -845,7 +864,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>46192</v>
       </c>
       <c r="B16" t="n">
@@ -871,7 +890,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="B17" t="n">
@@ -897,7 +916,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>46196</v>
       </c>
       <c r="B18" t="n">
@@ -923,7 +942,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>46197</v>
       </c>
       <c r="B19" t="n">
@@ -949,7 +968,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>46198</v>
       </c>
       <c r="B20" t="n">
@@ -975,7 +994,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="B21" t="n">
@@ -1001,7 +1020,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>46202</v>
       </c>
       <c r="B22" t="n">
@@ -1027,7 +1046,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="B23" t="n">
@@ -1066,7 +1085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1084,14 +1103,603 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>161.4922998677323</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>2026-06</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B3" t="n">
         <v>150.7558277000963</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Adj Close</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>VWAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B2" t="n">
+        <v>155.1610870361328</v>
+      </c>
+      <c r="C2" t="n">
+        <v>158</v>
+      </c>
+      <c r="D2" t="n">
+        <v>160.6999969482422</v>
+      </c>
+      <c r="E2" t="n">
+        <v>157.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>158.3000030517578</v>
+      </c>
+      <c r="G2" t="n">
+        <v>165375</v>
+      </c>
+      <c r="H2" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B3" t="n">
+        <v>155.9467163085938</v>
+      </c>
+      <c r="C3" t="n">
+        <v>158.8000030517578</v>
+      </c>
+      <c r="D3" t="n">
+        <v>160.1999969482422</v>
+      </c>
+      <c r="E3" t="n">
+        <v>155.3000030517578</v>
+      </c>
+      <c r="F3" t="n">
+        <v>158.3000030517578</v>
+      </c>
+      <c r="G3" t="n">
+        <v>200597</v>
+      </c>
+      <c r="H3" t="n">
+        <v>158.4384986069248</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B4" t="n">
+        <v>163.41015625</v>
+      </c>
+      <c r="C4" t="n">
+        <v>166.3999938964844</v>
+      </c>
+      <c r="D4" t="n">
+        <v>166.3999938964844</v>
+      </c>
+      <c r="E4" t="n">
+        <v>160.3999938964844</v>
+      </c>
+      <c r="F4" t="n">
+        <v>160.6000061035156</v>
+      </c>
+      <c r="G4" t="n">
+        <v>176050</v>
+      </c>
+      <c r="H4" t="n">
+        <v>161.02441070224</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B5" t="n">
+        <v>158.3035888671875</v>
+      </c>
+      <c r="C5" t="n">
+        <v>161.1999969482422</v>
+      </c>
+      <c r="D5" t="n">
+        <v>167.6000061035156</v>
+      </c>
+      <c r="E5" t="n">
+        <v>161.1999969482422</v>
+      </c>
+      <c r="F5" t="n">
+        <v>166.6999969482422</v>
+      </c>
+      <c r="G5" t="n">
+        <v>162765</v>
+      </c>
+      <c r="H5" t="n">
+        <v>161.0649609611559</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B6" t="n">
+        <v>159.8748474121094</v>
+      </c>
+      <c r="C6" t="n">
+        <v>162.8000030517578</v>
+      </c>
+      <c r="D6" t="n">
+        <v>163.3000030517578</v>
+      </c>
+      <c r="E6" t="n">
+        <v>159.8000030517578</v>
+      </c>
+      <c r="F6" t="n">
+        <v>160.3999938964844</v>
+      </c>
+      <c r="G6" t="n">
+        <v>96491</v>
+      </c>
+      <c r="H6" t="n">
+        <v>161.2738971185997</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B7" t="n">
+        <v>163.802978515625</v>
+      </c>
+      <c r="C7" t="n">
+        <v>166.8000030517578</v>
+      </c>
+      <c r="D7" t="n">
+        <v>166.8000030517578</v>
+      </c>
+      <c r="E7" t="n">
+        <v>162.3999938964844</v>
+      </c>
+      <c r="F7" t="n">
+        <v>162.8999938964844</v>
+      </c>
+      <c r="G7" t="n">
+        <v>195302</v>
+      </c>
+      <c r="H7" t="n">
+        <v>162.3568603939591</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B8" t="n">
+        <v>159.5802459716797</v>
+      </c>
+      <c r="C8" t="n">
+        <v>162.5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>166.3999938964844</v>
+      </c>
+      <c r="E8" t="n">
+        <v>161.3000030517578</v>
+      </c>
+      <c r="F8" t="n">
+        <v>165.3000030517578</v>
+      </c>
+      <c r="G8" t="n">
+        <v>118993</v>
+      </c>
+      <c r="H8" t="n">
+        <v>162.3721284321257</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B9" t="n">
+        <v>163.6065826416016</v>
+      </c>
+      <c r="C9" t="n">
+        <v>166.6000061035156</v>
+      </c>
+      <c r="D9" t="n">
+        <v>167.6999969482422</v>
+      </c>
+      <c r="E9" t="n">
+        <v>164.6999969482422</v>
+      </c>
+      <c r="F9" t="n">
+        <v>165.3999938964844</v>
+      </c>
+      <c r="G9" t="n">
+        <v>98127</v>
+      </c>
+      <c r="H9" t="n">
+        <v>162.7139500950246</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B10" t="n">
+        <v>164.8832092285156</v>
+      </c>
+      <c r="C10" t="n">
+        <v>167.8999938964844</v>
+      </c>
+      <c r="D10" t="n">
+        <v>169</v>
+      </c>
+      <c r="E10" t="n">
+        <v>165.8000030517578</v>
+      </c>
+      <c r="F10" t="n">
+        <v>168</v>
+      </c>
+      <c r="G10" t="n">
+        <v>70133</v>
+      </c>
+      <c r="H10" t="n">
+        <v>162.9972523702643</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B11" t="n">
+        <v>160.4640655517578</v>
+      </c>
+      <c r="C11" t="n">
+        <v>163.3999938964844</v>
+      </c>
+      <c r="D11" t="n">
+        <v>167.1000061035156</v>
+      </c>
+      <c r="E11" t="n">
+        <v>162.1999969482422</v>
+      </c>
+      <c r="F11" t="n">
+        <v>165.3999938964844</v>
+      </c>
+      <c r="G11" t="n">
+        <v>92390</v>
+      </c>
+      <c r="H11" t="n">
+        <v>163.0242896233893</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B12" t="n">
+        <v>157.0269470214844</v>
+      </c>
+      <c r="C12" t="n">
+        <v>159.8999938964844</v>
+      </c>
+      <c r="D12" t="n">
+        <v>163.3000030517578</v>
+      </c>
+      <c r="E12" t="n">
+        <v>159.1000061035156</v>
+      </c>
+      <c r="F12" t="n">
+        <v>161.6000061035156</v>
+      </c>
+      <c r="G12" t="n">
+        <v>124749</v>
+      </c>
+      <c r="H12" t="n">
+        <v>162.764622709126</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B13" t="n">
+        <v>151.5275726318359</v>
+      </c>
+      <c r="C13" t="n">
+        <v>154.3000030517578</v>
+      </c>
+      <c r="D13" t="n">
+        <v>160.1000061035156</v>
+      </c>
+      <c r="E13" t="n">
+        <v>153.3000030517578</v>
+      </c>
+      <c r="F13" t="n">
+        <v>158.6000061035156</v>
+      </c>
+      <c r="G13" t="n">
+        <v>135563</v>
+      </c>
+      <c r="H13" t="n">
+        <v>162.0634527160542</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B14" t="n">
+        <v>154.0808563232422</v>
+      </c>
+      <c r="C14" t="n">
+        <v>156.8999938964844</v>
+      </c>
+      <c r="D14" t="n">
+        <v>159</v>
+      </c>
+      <c r="E14" t="n">
+        <v>155</v>
+      </c>
+      <c r="F14" t="n">
+        <v>155</v>
+      </c>
+      <c r="G14" t="n">
+        <v>91945</v>
+      </c>
+      <c r="H14" t="n">
+        <v>161.788786985953</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B15" t="n">
+        <v>156.5359344482422</v>
+      </c>
+      <c r="C15" t="n">
+        <v>159.3999938964844</v>
+      </c>
+      <c r="D15" t="n">
+        <v>159.5</v>
+      </c>
+      <c r="E15" t="n">
+        <v>157.1000061035156</v>
+      </c>
+      <c r="F15" t="n">
+        <v>157.3999938964844</v>
+      </c>
+      <c r="G15" t="n">
+        <v>53036</v>
+      </c>
+      <c r="H15" t="n">
+        <v>161.7176722554128</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B16" t="n">
+        <v>158.5</v>
+      </c>
+      <c r="C16" t="n">
+        <v>161.3999938964844</v>
+      </c>
+      <c r="D16" t="n">
+        <v>162.8000030517578</v>
+      </c>
+      <c r="E16" t="n">
+        <v>160</v>
+      </c>
+      <c r="F16" t="n">
+        <v>161.5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>72064</v>
+      </c>
+      <c r="H16" t="n">
+        <v>161.7053214676087</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B17" t="n">
+        <v>162</v>
+      </c>
+      <c r="C17" t="n">
+        <v>162</v>
+      </c>
+      <c r="D17" t="n">
+        <v>162.5</v>
+      </c>
+      <c r="E17" t="n">
+        <v>160.6999969482422</v>
+      </c>
+      <c r="F17" t="n">
+        <v>161.6000061035156</v>
+      </c>
+      <c r="G17" t="n">
+        <v>69509</v>
+      </c>
+      <c r="H17" t="n">
+        <v>161.7159724619766</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>46168</v>
+      </c>
+      <c r="B18" t="n">
+        <v>161.6000061035156</v>
+      </c>
+      <c r="C18" t="n">
+        <v>161.6000061035156</v>
+      </c>
+      <c r="D18" t="n">
+        <v>164.1999969482422</v>
+      </c>
+      <c r="E18" t="n">
+        <v>160.6999969482422</v>
+      </c>
+      <c r="F18" t="n">
+        <v>161.8999938964844</v>
+      </c>
+      <c r="G18" t="n">
+        <v>107500</v>
+      </c>
+      <c r="H18" t="n">
+        <v>161.7098331676465</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B19" t="n">
+        <v>161</v>
+      </c>
+      <c r="C19" t="n">
+        <v>161</v>
+      </c>
+      <c r="D19" t="n">
+        <v>164.3000030517578</v>
+      </c>
+      <c r="E19" t="n">
+        <v>159.3999938964844</v>
+      </c>
+      <c r="F19" t="n">
+        <v>162.1999969482422</v>
+      </c>
+      <c r="G19" t="n">
+        <v>92700</v>
+      </c>
+      <c r="H19" t="n">
+        <v>161.6788427868548</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B20" t="n">
+        <v>162.6000061035156</v>
+      </c>
+      <c r="C20" t="n">
+        <v>162.6000061035156</v>
+      </c>
+      <c r="D20" t="n">
+        <v>162.6000061035156</v>
+      </c>
+      <c r="E20" t="n">
+        <v>158.3000030517578</v>
+      </c>
+      <c r="F20" t="n">
+        <v>161.1000061035156</v>
+      </c>
+      <c r="G20" t="n">
+        <v>110364</v>
+      </c>
+      <c r="H20" t="n">
+        <v>161.7243571385826</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B21" t="n">
+        <v>158.3999938964844</v>
+      </c>
+      <c r="C21" t="n">
+        <v>158.3999938964844</v>
+      </c>
+      <c r="D21" t="n">
+        <v>163</v>
+      </c>
+      <c r="E21" t="n">
+        <v>158</v>
+      </c>
+      <c r="F21" t="n">
+        <v>163</v>
+      </c>
+      <c r="G21" t="n">
+        <v>167621</v>
+      </c>
+      <c r="H21" t="n">
+        <v>161.4922998677323</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>